<commit_message>
feat: implement big matrix Excel report generation and add application core structure
</commit_message>
<xml_diff>
--- a/bomix-app/backend/excel/template/bigmatrix.xlsx
+++ b/bomix-app/backend/excel/template/bigmatrix.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\Programming\BOMIX\bomix-app\backend\excel\template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F892BB7D-38BC-4153-B75B-268FCD1456B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81E87ED6-9CA3-4763-A027-F37469110B88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="76680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B3540397-11C0-482D-9795-221357CC67A7}"/>
+    <workbookView xWindow="30756" yWindow="4800" windowWidth="28056" windowHeight="17772" xr2:uid="{B3540397-11C0-482D-9795-221357CC67A7}"/>
   </bookViews>
   <sheets>
     <sheet name="BigMatrix" sheetId="2" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="27">
   <si>
     <t>Item</t>
   </si>
@@ -81,9 +81,6 @@
   </si>
   <si>
     <t>AD3</t>
-  </si>
-  <si>
-    <t>V</t>
   </si>
   <si>
     <t>A</t>
@@ -209,7 +206,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="13">
+  <borders count="14">
     <border>
       <left/>
       <right/>
@@ -393,15 +390,21 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="centerContinuous" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -412,30 +415,12 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -465,28 +450,61 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -504,10 +522,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -801,7 +815,7 @@
   <sheetFormatPr defaultRowHeight="13.2"/>
   <cols>
     <col min="1" max="1" width="4.6640625" customWidth="1"/>
-    <col min="2" max="2" width="14.6640625" customWidth="1"/>
+    <col min="2" max="2" width="14.6640625" style="26" customWidth="1"/>
     <col min="3" max="3" width="35.88671875" customWidth="1"/>
     <col min="4" max="4" width="10.6640625" customWidth="1"/>
     <col min="5" max="5" width="17.6640625" customWidth="1"/>
@@ -811,156 +825,154 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10">
-      <c r="A1" s="1"/>
-      <c r="B1" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
+      <c r="A1" s="27" t="s">
+        <v>24</v>
+      </c>
+      <c r="B1" s="27"/>
+      <c r="C1" s="27"/>
+      <c r="D1" s="27"/>
+      <c r="E1" s="27"/>
+      <c r="F1" s="27"/>
+      <c r="G1" s="27"/>
     </row>
     <row r="2" spans="1:10">
-      <c r="A2" s="1"/>
-      <c r="B2" s="1" t="s">
+      <c r="A2" s="27" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="1"/>
-      <c r="D2" s="1"/>
-      <c r="E2" s="1"/>
-      <c r="F2" s="1"/>
-      <c r="G2" s="1"/>
-      <c r="H2" s="28" t="s">
-        <v>26</v>
-      </c>
-      <c r="I2" s="29"/>
-      <c r="J2" s="30"/>
+      <c r="B2" s="27"/>
+      <c r="C2" s="27"/>
+      <c r="D2" s="27"/>
+      <c r="E2" s="27"/>
+      <c r="F2" s="27"/>
+      <c r="G2" s="28"/>
+      <c r="H2" s="19" t="s">
+        <v>25</v>
+      </c>
+      <c r="I2" s="20"/>
+      <c r="J2" s="21"/>
     </row>
     <row r="3" spans="1:10">
-      <c r="A3" s="2"/>
-      <c r="B3" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="C3" s="2"/>
-      <c r="D3" s="2"/>
-      <c r="E3" s="2"/>
-      <c r="F3" s="2"/>
-      <c r="G3" s="2"/>
-      <c r="H3" s="25" t="s">
-        <v>20</v>
-      </c>
-      <c r="I3" s="26"/>
-      <c r="J3" s="27"/>
+      <c r="A3" s="1"/>
+      <c r="B3" s="22" t="s">
+        <v>23</v>
+      </c>
+      <c r="C3" s="1"/>
+      <c r="D3" s="1"/>
+      <c r="E3" s="1"/>
+      <c r="F3" s="1"/>
+      <c r="G3" s="1"/>
+      <c r="H3" s="16" t="s">
+        <v>19</v>
+      </c>
+      <c r="I3" s="17"/>
+      <c r="J3" s="18"/>
     </row>
     <row r="4" spans="1:10">
-      <c r="A4" s="2"/>
-      <c r="B4" s="2" t="s">
+      <c r="A4" s="1"/>
+      <c r="B4" s="22" t="s">
+        <v>21</v>
+      </c>
+      <c r="C4" s="1"/>
+      <c r="D4" s="1"/>
+      <c r="E4" s="1"/>
+      <c r="F4" s="1"/>
+      <c r="G4" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="C4" s="2"/>
-      <c r="D4" s="2"/>
-      <c r="E4" s="2"/>
-      <c r="F4" s="2"/>
-      <c r="G4" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="H4" s="15" t="s">
+      <c r="H4" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="I4" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="I4" s="3" t="s">
+      <c r="J4" s="9" t="s">
         <v>18</v>
-      </c>
-      <c r="J4" s="16" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="5" spans="1:10">
-      <c r="A5" s="3" t="s">
+      <c r="A5" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B5" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="C5" s="3" t="s">
+      <c r="B5" s="23" t="s">
+        <v>20</v>
+      </c>
+      <c r="C5" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="D5" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="E5" s="3" t="s">
+      <c r="E5" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="F5" s="3" t="s">
+      <c r="F5" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="G5" s="14" t="s">
+      <c r="G5" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="H5" s="17"/>
-      <c r="I5" s="4"/>
-      <c r="J5" s="20"/>
+      <c r="H5" s="10"/>
+      <c r="I5" s="3"/>
+      <c r="J5" s="13"/>
     </row>
     <row r="6" spans="1:10" ht="20.399999999999999">
-      <c r="A6" s="6">
+      <c r="A6" s="4">
         <v>31</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="B6" s="24" t="s">
         <v>7</v>
       </c>
-      <c r="C6" s="7" t="s">
+      <c r="C6" s="29" t="s">
         <v>8</v>
       </c>
-      <c r="D6" s="5" t="s">
+      <c r="D6" s="24" t="s">
         <v>9</v>
       </c>
-      <c r="E6" s="7" t="s">
+      <c r="E6" s="29" t="s">
         <v>10</v>
       </c>
-      <c r="F6" s="6">
+      <c r="F6" s="4">
         <v>5</v>
       </c>
-      <c r="G6" s="23" t="s">
+      <c r="G6" s="32" t="s">
         <v>11</v>
       </c>
-      <c r="H6" s="18" t="s">
-        <v>16</v>
-      </c>
-      <c r="I6" s="12"/>
-      <c r="J6" s="22"/>
+      <c r="H6" s="11"/>
+      <c r="I6" s="6"/>
+      <c r="J6" s="15"/>
     </row>
     <row r="7" spans="1:10" ht="40.799999999999997">
-      <c r="A7" s="9">
+      <c r="A7" s="5">
         <v>32</v>
       </c>
-      <c r="B7" s="8" t="s">
+      <c r="B7" s="25" t="s">
         <v>12</v>
       </c>
-      <c r="C7" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="D7" s="8" t="s">
+      <c r="C7" s="30" t="s">
+        <v>26</v>
+      </c>
+      <c r="D7" s="25" t="s">
         <v>13</v>
       </c>
-      <c r="E7" s="10" t="s">
+      <c r="E7" s="31" t="s">
         <v>14</v>
       </c>
-      <c r="F7" s="9">
+      <c r="F7" s="5">
         <v>1</v>
       </c>
-      <c r="G7" s="24" t="s">
+      <c r="G7" s="33" t="s">
         <v>15</v>
       </c>
-      <c r="H7" s="19" t="s">
-        <v>16</v>
-      </c>
-      <c r="I7" s="13"/>
-      <c r="J7" s="21"/>
+      <c r="H7" s="12"/>
+      <c r="I7" s="34"/>
+      <c r="J7" s="14"/>
     </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="4">
     <mergeCell ref="H3:J3"/>
     <mergeCell ref="H2:J2"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A2:G2"/>
   </mergeCells>
   <phoneticPr fontId="5" type="noConversion"/>
   <printOptions gridLinesSet="0"/>

</xml_diff>

<commit_message>
feat: implement BigMatrix excel writer with template support and data processing utilities
</commit_message>
<xml_diff>
--- a/bomix-app/backend/excel/template/bigmatrix.xlsx
+++ b/bomix-app/backend/excel/template/bigmatrix.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\Programming\BOMIX\bomix-app\backend\excel\template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81E87ED6-9CA3-4763-A027-F37469110B88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A586D3EB-426C-4A46-9997-15EC09015AC4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="30756" yWindow="4800" windowWidth="28056" windowHeight="17772" xr2:uid="{B3540397-11C0-482D-9795-221357CC67A7}"/>
+    <workbookView xWindow="23124" yWindow="3972" windowWidth="23016" windowHeight="20064" xr2:uid="{B3540397-11C0-482D-9795-221357CC67A7}"/>
   </bookViews>
   <sheets>
     <sheet name="BigMatrix" sheetId="2" r:id="rId1"/>
@@ -403,7 +403,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -450,30 +450,9 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -483,12 +462,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -505,6 +478,30 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -815,7 +812,7 @@
   <sheetFormatPr defaultRowHeight="13.2"/>
   <cols>
     <col min="1" max="1" width="4.6640625" customWidth="1"/>
-    <col min="2" max="2" width="14.6640625" style="26" customWidth="1"/>
+    <col min="2" max="2" width="14.6640625" style="19" customWidth="1"/>
     <col min="3" max="3" width="35.88671875" customWidth="1"/>
     <col min="4" max="4" width="10.6640625" customWidth="1"/>
     <col min="5" max="5" width="17.6640625" customWidth="1"/>
@@ -825,35 +822,35 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10">
-      <c r="A1" s="27" t="s">
+      <c r="A1" s="32" t="s">
         <v>24</v>
       </c>
-      <c r="B1" s="27"/>
-      <c r="C1" s="27"/>
-      <c r="D1" s="27"/>
-      <c r="E1" s="27"/>
-      <c r="F1" s="27"/>
-      <c r="G1" s="27"/>
+      <c r="B1" s="32"/>
+      <c r="C1" s="32"/>
+      <c r="D1" s="32"/>
+      <c r="E1" s="32"/>
+      <c r="F1" s="32"/>
+      <c r="G1" s="32"/>
     </row>
     <row r="2" spans="1:10">
-      <c r="A2" s="27" t="s">
+      <c r="A2" s="32" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="27"/>
-      <c r="C2" s="27"/>
-      <c r="D2" s="27"/>
-      <c r="E2" s="27"/>
-      <c r="F2" s="27"/>
-      <c r="G2" s="28"/>
-      <c r="H2" s="19" t="s">
+      <c r="B2" s="32"/>
+      <c r="C2" s="32"/>
+      <c r="D2" s="32"/>
+      <c r="E2" s="32"/>
+      <c r="F2" s="32"/>
+      <c r="G2" s="33"/>
+      <c r="H2" s="29" t="s">
         <v>25</v>
       </c>
-      <c r="I2" s="20"/>
-      <c r="J2" s="21"/>
+      <c r="I2" s="30"/>
+      <c r="J2" s="31"/>
     </row>
     <row r="3" spans="1:10">
       <c r="A3" s="1"/>
-      <c r="B3" s="22" t="s">
+      <c r="B3" s="16" t="s">
         <v>23</v>
       </c>
       <c r="C3" s="1"/>
@@ -861,15 +858,15 @@
       <c r="E3" s="1"/>
       <c r="F3" s="1"/>
       <c r="G3" s="1"/>
-      <c r="H3" s="16" t="s">
+      <c r="H3" s="26" t="s">
         <v>19</v>
       </c>
-      <c r="I3" s="17"/>
-      <c r="J3" s="18"/>
+      <c r="I3" s="27"/>
+      <c r="J3" s="28"/>
     </row>
     <row r="4" spans="1:10">
       <c r="A4" s="1"/>
-      <c r="B4" s="22" t="s">
+      <c r="B4" s="16" t="s">
         <v>21</v>
       </c>
       <c r="C4" s="1"/>
@@ -893,7 +890,7 @@
       <c r="A5" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B5" s="23" t="s">
+      <c r="B5" s="2" t="s">
         <v>20</v>
       </c>
       <c r="C5" s="2" t="s">
@@ -919,22 +916,22 @@
       <c r="A6" s="4">
         <v>31</v>
       </c>
-      <c r="B6" s="24" t="s">
+      <c r="B6" s="17" t="s">
         <v>7</v>
       </c>
-      <c r="C6" s="29" t="s">
+      <c r="C6" s="20" t="s">
         <v>8</v>
       </c>
-      <c r="D6" s="24" t="s">
+      <c r="D6" s="17" t="s">
         <v>9</v>
       </c>
-      <c r="E6" s="29" t="s">
+      <c r="E6" s="20" t="s">
         <v>10</v>
       </c>
       <c r="F6" s="4">
         <v>5</v>
       </c>
-      <c r="G6" s="32" t="s">
+      <c r="G6" s="23" t="s">
         <v>11</v>
       </c>
       <c r="H6" s="11"/>
@@ -945,26 +942,26 @@
       <c r="A7" s="5">
         <v>32</v>
       </c>
-      <c r="B7" s="25" t="s">
+      <c r="B7" s="18" t="s">
         <v>12</v>
       </c>
-      <c r="C7" s="30" t="s">
+      <c r="C7" s="21" t="s">
         <v>26</v>
       </c>
-      <c r="D7" s="25" t="s">
+      <c r="D7" s="18" t="s">
         <v>13</v>
       </c>
-      <c r="E7" s="31" t="s">
+      <c r="E7" s="22" t="s">
         <v>14</v>
       </c>
       <c r="F7" s="5">
         <v>1</v>
       </c>
-      <c r="G7" s="33" t="s">
+      <c r="G7" s="24" t="s">
         <v>15</v>
       </c>
       <c r="H7" s="12"/>
-      <c r="I7" s="34"/>
+      <c r="I7" s="25"/>
       <c r="J7" s="14"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
修正matrix model name 流程
</commit_message>
<xml_diff>
--- a/bomix-app/backend/excel/template/bigmatrix.xlsx
+++ b/bomix-app/backend/excel/template/bigmatrix.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\Programming\BOMIX\bomix-app\backend\excel\template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27F71426-3C23-4AFB-B315-185314527B08}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B54A7650-B08A-4051-964D-78F01422B323}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6300" yWindow="4656" windowWidth="29856" windowHeight="20400" xr2:uid="{B3540397-11C0-482D-9795-221357CC67A7}"/>
+    <workbookView xWindow="7164" yWindow="1188" windowWidth="36288" windowHeight="22500" xr2:uid="{B3540397-11C0-482D-9795-221357CC67A7}"/>
   </bookViews>
   <sheets>
     <sheet name="BigMatrix" sheetId="2" r:id="rId1"/>
@@ -95,10 +95,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>PV-0.3</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>HH PN</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -119,11 +115,15 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>Taris</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>TVS-Array,Ir(max)=1uA,Vc(max)=8V@Ipp=5A,Vrwm(max)=3.3V,Vbr(min)=4V,16KV(air),16KV(contact),DFN1006-2P,SMD,ROHS,HF</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>TestProj</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>DB-0.9</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -405,37 +405,13 @@
   </cellStyleXfs>
   <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -492,6 +468,30 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -800,159 +800,159 @@
   <dimension ref="A1:J7"/>
   <sheetFormatPr defaultRowHeight="13.8"/>
   <cols>
-    <col min="1" max="1" width="4.6640625" style="2" customWidth="1"/>
-    <col min="2" max="2" width="14.6640625" style="30" customWidth="1"/>
-    <col min="3" max="3" width="35.88671875" style="2" customWidth="1"/>
-    <col min="4" max="4" width="10.6640625" style="2" customWidth="1"/>
-    <col min="5" max="5" width="17.6640625" style="2" customWidth="1"/>
-    <col min="6" max="6" width="4.6640625" style="2" customWidth="1"/>
-    <col min="7" max="7" width="18.6640625" style="2" customWidth="1"/>
-    <col min="8" max="10" width="2.88671875" style="2" bestFit="1" customWidth="1"/>
-    <col min="11" max="16384" width="8.88671875" style="2"/>
+    <col min="1" max="1" width="4.6640625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="14.6640625" style="22" customWidth="1"/>
+    <col min="3" max="3" width="35.88671875" style="1" customWidth="1"/>
+    <col min="4" max="4" width="10.6640625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="17.6640625" style="1" customWidth="1"/>
+    <col min="6" max="6" width="4.6640625" style="1" customWidth="1"/>
+    <col min="7" max="7" width="18.6640625" style="1" customWidth="1"/>
+    <col min="8" max="10" width="2.88671875" style="1" bestFit="1" customWidth="1"/>
+    <col min="11" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10">
-      <c r="A1" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
+      <c r="A1" s="29" t="s">
+        <v>23</v>
+      </c>
+      <c r="B1" s="29"/>
+      <c r="C1" s="29"/>
+      <c r="D1" s="29"/>
+      <c r="E1" s="29"/>
+      <c r="F1" s="29"/>
+      <c r="G1" s="29"/>
     </row>
     <row r="2" spans="1:10">
-      <c r="A2" s="1" t="s">
+      <c r="A2" s="29" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="1"/>
-      <c r="C2" s="1"/>
-      <c r="D2" s="1"/>
-      <c r="E2" s="1"/>
-      <c r="F2" s="1"/>
-      <c r="G2" s="3"/>
-      <c r="H2" s="4" t="s">
+      <c r="B2" s="29"/>
+      <c r="C2" s="29"/>
+      <c r="D2" s="29"/>
+      <c r="E2" s="29"/>
+      <c r="F2" s="29"/>
+      <c r="G2" s="30"/>
+      <c r="H2" s="26" t="s">
         <v>25</v>
       </c>
-      <c r="I2" s="5"/>
-      <c r="J2" s="6"/>
+      <c r="I2" s="27"/>
+      <c r="J2" s="28"/>
     </row>
     <row r="3" spans="1:10">
-      <c r="A3" s="7"/>
-      <c r="B3" s="8" t="s">
-        <v>23</v>
-      </c>
-      <c r="C3" s="7"/>
-      <c r="D3" s="7"/>
-      <c r="E3" s="7"/>
-      <c r="F3" s="7"/>
-      <c r="G3" s="7"/>
-      <c r="H3" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="I3" s="10"/>
-      <c r="J3" s="11"/>
+      <c r="A3" s="2"/>
+      <c r="B3" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2"/>
+      <c r="F3" s="2"/>
+      <c r="G3" s="2"/>
+      <c r="H3" s="23" t="s">
+        <v>26</v>
+      </c>
+      <c r="I3" s="24"/>
+      <c r="J3" s="25"/>
     </row>
     <row r="4" spans="1:10">
-      <c r="A4" s="7"/>
-      <c r="B4" s="8" t="s">
+      <c r="A4" s="2"/>
+      <c r="B4" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="C4" s="2"/>
+      <c r="D4" s="2"/>
+      <c r="E4" s="2"/>
+      <c r="F4" s="2"/>
+      <c r="G4" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C4" s="7"/>
-      <c r="D4" s="7"/>
-      <c r="E4" s="7"/>
-      <c r="F4" s="7"/>
-      <c r="G4" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="H4" s="12" t="s">
+      <c r="H4" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="I4" s="13" t="s">
+      <c r="I4" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="J4" s="14" t="s">
+      <c r="J4" s="6" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="5" spans="1:10">
-      <c r="A5" s="13" t="s">
+      <c r="A5" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B5" s="13" t="s">
-        <v>20</v>
-      </c>
-      <c r="C5" s="13" t="s">
+      <c r="B5" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="C5" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="D5" s="13" t="s">
+      <c r="D5" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="E5" s="13" t="s">
+      <c r="E5" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="F5" s="13" t="s">
+      <c r="F5" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="G5" s="15" t="s">
+      <c r="G5" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="H5" s="16"/>
-      <c r="I5" s="17"/>
-      <c r="J5" s="18"/>
+      <c r="H5" s="8"/>
+      <c r="I5" s="9"/>
+      <c r="J5" s="10"/>
     </row>
     <row r="6" spans="1:10" ht="20.399999999999999">
-      <c r="A6" s="19">
+      <c r="A6" s="11">
         <v>31</v>
       </c>
-      <c r="B6" s="20" t="s">
+      <c r="B6" s="12" t="s">
         <v>7</v>
       </c>
-      <c r="C6" s="21" t="s">
+      <c r="C6" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="D6" s="20" t="s">
+      <c r="D6" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="E6" s="21" t="s">
+      <c r="E6" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="F6" s="19">
+      <c r="F6" s="11">
         <v>5</v>
       </c>
-      <c r="G6" s="22" t="s">
+      <c r="G6" s="14" t="s">
         <v>11</v>
       </c>
-      <c r="H6" s="16"/>
-      <c r="I6" s="17"/>
-      <c r="J6" s="18"/>
+      <c r="H6" s="8"/>
+      <c r="I6" s="9"/>
+      <c r="J6" s="10"/>
     </row>
     <row r="7" spans="1:10" ht="40.799999999999997">
-      <c r="A7" s="23">
+      <c r="A7" s="15">
         <v>32</v>
       </c>
-      <c r="B7" s="24" t="s">
+      <c r="B7" s="16" t="s">
         <v>12</v>
       </c>
-      <c r="C7" s="25" t="s">
-        <v>26</v>
-      </c>
-      <c r="D7" s="24" t="s">
+      <c r="C7" s="17" t="s">
+        <v>24</v>
+      </c>
+      <c r="D7" s="16" t="s">
         <v>13</v>
       </c>
-      <c r="E7" s="25" t="s">
+      <c r="E7" s="17" t="s">
         <v>14</v>
       </c>
-      <c r="F7" s="23">
+      <c r="F7" s="15">
         <v>1</v>
       </c>
-      <c r="G7" s="26" t="s">
+      <c r="G7" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="H7" s="27"/>
-      <c r="I7" s="28"/>
-      <c r="J7" s="29"/>
+      <c r="H7" s="19"/>
+      <c r="I7" s="20"/>
+      <c r="J7" s="21"/>
     </row>
   </sheetData>
   <mergeCells count="4">

</xml_diff>